<commit_message>
ManagmentSustem event function configured
</commit_message>
<xml_diff>
--- a/TODO_List.xlsx
+++ b/TODO_List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clash\CourseWork\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105DF32D-9428-422C-A780-BD3D22B65A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D6474C-F98D-45C8-B086-90EE231B4F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Task</t>
   </si>
@@ -37,6 +37,12 @@
   </si>
   <si>
     <t>"Models" correction</t>
+  </si>
+  <si>
+    <t>FACADE for MainService</t>
+  </si>
+  <si>
+    <t>№</t>
   </si>
 </sst>
 </file>
@@ -387,13 +393,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="G11:H15"/>
+  <dimension ref="F11:H15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="7:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F11" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G11" s="2" t="s">
         <v>0</v>
       </c>
@@ -401,23 +410,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="7:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
       <c r="G12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="7:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F13" s="1">
+        <v>2</v>
+      </c>
       <c r="G13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G14" s="1"/>
+    <row r="14" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F14" s="1">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="7:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="6:8" x14ac:dyDescent="0.25">
+      <c r="F15" s="1">
+        <v>4</v>
+      </c>
       <c r="G15" s="1"/>
       <c r="H15" s="3"/>
     </row>

</xml_diff>

<commit_message>
Registration Window, and VM were added to rep
</commit_message>
<xml_diff>
--- a/TODO_List.xlsx
+++ b/TODO_List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clash\CourseWork\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D6474C-F98D-45C8-B086-90EE231B4F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8342B12-E16B-4EC5-A40F-6FAAF83B3BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,10 +49,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -105,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -113,6 +120,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,7 +443,7 @@
       <c r="G14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H14" s="3"/>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F15" s="1">

</xml_diff>